<commit_message>
Updates for Ubuntu run
</commit_message>
<xml_diff>
--- a/mcp-manual-test-sheet.xlsx
+++ b/mcp-manual-test-sheet.xlsx
@@ -1045,7 +1045,7 @@
         </is>
       </c>
       <c r="E21" s="13">
-        <f>"U='"&amp;$B$7&amp;"/wp-admin/admin.php?page="&amp;$B$4&amp;"'; open ""$U"" 2&gt;/dev/null || xdg-open ""$U"""</f>
+        <f>"U='"&amp;$B$7&amp;"/wp-admin/admin.php?page="&amp;$B$4&amp;"'; xdg-open ""$U"" 2&gt;/dev/null || open ""$U"""</f>
         <v/>
       </c>
       <c r="F21" s="12" t="inlineStr">
@@ -1579,7 +1579,7 @@
         </is>
       </c>
       <c r="E40" s="13">
-        <f>"for U in 'https://wordpress.org/support/plugin/"&amp;$B$4&amp;"/' 'https://wordpress.org/plugins/"&amp;$B$4&amp;"/#description'; do open ""$U"" 2&gt;/dev/null || xdg-open ""$U""; done"</f>
+        <f>"for U in 'https://wordpress.org/support/plugin/"&amp;$B$4&amp;"/' 'https://wordpress.org/plugins/"&amp;$B$4&amp;"/#description'; do xdg-open ""$U"" 2&gt;/dev/null || open ""$U""; done"</f>
         <v/>
       </c>
       <c r="F40" s="12" t="inlineStr">

</xml_diff>